<commit_message>
Translate Excel files to English, rebrand OLADE to OSTRAM, and auto-discover scenarios
- Rename OLADE Excel files to OSTRAM naming convention and translate all
  Spanish technology/fuel names to English across 4 Excel files
- Replace Latin American countries with South Asian region (Bangladesh,
  Bhutan, India, Maldives, Nepal, Sri Lanka) in data Excel files
- Replace all OLADE references with OSTRAM across D1, D2, config loader,
  and country codes YAML
- Remove hardcoded scenario lists in D1_generate_editor_template.py,
  replacing them with auto-discovery from A1_Outputs_* folders
- Improve documentation with pipeline clarifications and comment out
  Auxiliary Tools section
</commit_message>
<xml_diff>
--- a/t1_confection/A1_Outputs/A1_Outputs_BAU/A-O_Demand.xlsx
+++ b/t1_confection/A1_Outputs/A1_Outputs_BAU/A-O_Demand.xlsx
@@ -502,7 +502,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ11"/>
+  <dimension ref="A1:AJ12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13.85546875" bestFit="1" customWidth="1" style="4" min="1" max="1"/>
@@ -738,88 +738,88 @@
         <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>499.71</v>
+        <v>469.23</v>
       </c>
       <c r="J2" t="n">
-        <v>542.73</v>
+        <v>478.61</v>
       </c>
       <c r="K2" t="n">
-        <v>585.75</v>
+        <v>488</v>
       </c>
       <c r="L2" t="n">
-        <v>631.35</v>
+        <v>497.38</v>
       </c>
       <c r="M2" t="n">
-        <v>676.95</v>
+        <v>506.77</v>
       </c>
       <c r="N2" t="n">
-        <v>722.54</v>
+        <v>516.15</v>
       </c>
       <c r="O2" t="n">
-        <v>768.14</v>
+        <v>525.54</v>
       </c>
       <c r="P2" t="n">
-        <v>813.74</v>
+        <v>534.92</v>
       </c>
       <c r="Q2" t="n">
-        <v>860.42</v>
+        <v>544.3099999999999</v>
       </c>
       <c r="R2" t="n">
-        <v>907.11</v>
+        <v>553.6900000000001</v>
       </c>
       <c r="S2" t="n">
-        <v>953.79</v>
+        <v>563.08</v>
       </c>
       <c r="T2" t="n">
-        <v>1000.48</v>
+        <v>572.46</v>
       </c>
       <c r="U2" t="n">
-        <v>1047.16</v>
+        <v>581.85</v>
       </c>
       <c r="V2" t="n">
-        <v>1094.98</v>
+        <v>591.23</v>
       </c>
       <c r="W2" t="n">
-        <v>1142.8</v>
+        <v>600.61</v>
       </c>
       <c r="X2" t="n">
-        <v>1190.62</v>
+        <v>610</v>
       </c>
       <c r="Y2" t="n">
-        <v>1238.44</v>
+        <v>619.38</v>
       </c>
       <c r="Z2" t="n">
-        <v>1286.25</v>
+        <v>628.77</v>
       </c>
       <c r="AA2" t="n">
-        <v>1334.01</v>
+        <v>638.15</v>
       </c>
       <c r="AB2" t="n">
-        <v>1381.76</v>
+        <v>647.54</v>
       </c>
       <c r="AC2" t="n">
-        <v>1429.51</v>
+        <v>656.92</v>
       </c>
       <c r="AD2" t="n">
-        <v>1477.26</v>
+        <v>666.3099999999999</v>
       </c>
       <c r="AE2" t="n">
-        <v>1525.02</v>
+        <v>675.6900000000001</v>
       </c>
       <c r="AF2" t="n">
-        <v>1574.01</v>
+        <v>685.08</v>
       </c>
       <c r="AG2" t="n">
-        <v>1623.01</v>
+        <v>694.46</v>
       </c>
       <c r="AH2" t="n">
-        <v>1672</v>
+        <v>703.85</v>
       </c>
       <c r="AI2" t="n">
-        <v>1721</v>
+        <v>713.23</v>
       </c>
       <c r="AJ2" t="n">
-        <v>1769.99</v>
+        <v>722.61</v>
       </c>
     </row>
     <row r="3">
@@ -862,88 +862,88 @@
         <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>12.58</v>
+        <v>3.87</v>
       </c>
       <c r="J3" t="n">
-        <v>14.11</v>
+        <v>3.95</v>
       </c>
       <c r="K3" t="n">
-        <v>15.66</v>
+        <v>4.03</v>
       </c>
       <c r="L3" t="n">
-        <v>17.32</v>
+        <v>4.11</v>
       </c>
       <c r="M3" t="n">
-        <v>18.97</v>
+        <v>4.18</v>
       </c>
       <c r="N3" t="n">
-        <v>20.62</v>
+        <v>4.26</v>
       </c>
       <c r="O3" t="n">
-        <v>22.27</v>
+        <v>4.34</v>
       </c>
       <c r="P3" t="n">
-        <v>23.95</v>
+        <v>4.42</v>
       </c>
       <c r="Q3" t="n">
-        <v>25.73</v>
+        <v>4.49</v>
       </c>
       <c r="R3" t="n">
-        <v>27.51</v>
+        <v>4.57</v>
       </c>
       <c r="S3" t="n">
-        <v>29.28</v>
+        <v>4.65</v>
       </c>
       <c r="T3" t="n">
-        <v>31.09</v>
+        <v>4.73</v>
       </c>
       <c r="U3" t="n">
-        <v>32.86</v>
+        <v>4.8</v>
       </c>
       <c r="V3" t="n">
-        <v>34.84</v>
+        <v>4.88</v>
       </c>
       <c r="W3" t="n">
-        <v>36.82</v>
+        <v>4.96</v>
       </c>
       <c r="X3" t="n">
-        <v>38.8</v>
+        <v>5.04</v>
       </c>
       <c r="Y3" t="n">
-        <v>40.78</v>
+        <v>5.11</v>
       </c>
       <c r="Z3" t="n">
-        <v>42.75</v>
+        <v>5.19</v>
       </c>
       <c r="AA3" t="n">
-        <v>44.93</v>
+        <v>5.27</v>
       </c>
       <c r="AB3" t="n">
-        <v>47.11</v>
+        <v>5.35</v>
       </c>
       <c r="AC3" t="n">
-        <v>49.29</v>
+        <v>5.42</v>
       </c>
       <c r="AD3" t="n">
-        <v>51.47</v>
+        <v>5.5</v>
       </c>
       <c r="AE3" t="n">
-        <v>53.64</v>
+        <v>5.58</v>
       </c>
       <c r="AF3" t="n">
-        <v>56</v>
+        <v>5.66</v>
       </c>
       <c r="AG3" t="n">
-        <v>58.35</v>
+        <v>5.73</v>
       </c>
       <c r="AH3" t="n">
-        <v>60.7</v>
+        <v>5.81</v>
       </c>
       <c r="AI3" t="n">
-        <v>63.06</v>
+        <v>5.89</v>
       </c>
       <c r="AJ3" t="n">
-        <v>65.41</v>
+        <v>5.97</v>
       </c>
     </row>
     <row r="4">
@@ -1606,88 +1606,88 @@
         <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>47.48</v>
+        <v>290.09</v>
       </c>
       <c r="J9" t="n">
-        <v>47.48</v>
+        <v>295.89</v>
       </c>
       <c r="K9" t="n">
-        <v>47.48</v>
+        <v>301.69</v>
       </c>
       <c r="L9" t="n">
-        <v>54.22</v>
+        <v>307.49</v>
       </c>
       <c r="M9" t="n">
-        <v>60.95</v>
+        <v>313.3</v>
       </c>
       <c r="N9" t="n">
-        <v>67.69</v>
+        <v>319.1</v>
       </c>
       <c r="O9" t="n">
-        <v>74.42</v>
+        <v>324.9</v>
       </c>
       <c r="P9" t="n">
-        <v>81.15000000000001</v>
+        <v>330.7</v>
       </c>
       <c r="Q9" t="n">
-        <v>88.8</v>
+        <v>336.5</v>
       </c>
       <c r="R9" t="n">
-        <v>96.45999999999999</v>
+        <v>342.31</v>
       </c>
       <c r="S9" t="n">
-        <v>104.11</v>
+        <v>348.11</v>
       </c>
       <c r="T9" t="n">
-        <v>111.76</v>
+        <v>353.91</v>
       </c>
       <c r="U9" t="n">
-        <v>119.41</v>
+        <v>359.71</v>
       </c>
       <c r="V9" t="n">
-        <v>127.6</v>
+        <v>365.51</v>
       </c>
       <c r="W9" t="n">
-        <v>135.78</v>
+        <v>371.31</v>
       </c>
       <c r="X9" t="n">
-        <v>143.96</v>
+        <v>377.12</v>
       </c>
       <c r="Y9" t="n">
-        <v>152.15</v>
+        <v>382.92</v>
       </c>
       <c r="Z9" t="n">
-        <v>160.33</v>
+        <v>388.72</v>
       </c>
       <c r="AA9" t="n">
-        <v>168.97</v>
+        <v>394.52</v>
       </c>
       <c r="AB9" t="n">
-        <v>177.6</v>
+        <v>400.32</v>
       </c>
       <c r="AC9" t="n">
-        <v>186.23</v>
+        <v>406.13</v>
       </c>
       <c r="AD9" t="n">
-        <v>194.87</v>
+        <v>411.93</v>
       </c>
       <c r="AE9" t="n">
-        <v>203.5</v>
+        <v>417.73</v>
       </c>
       <c r="AF9" t="n">
-        <v>212.6</v>
+        <v>423.53</v>
       </c>
       <c r="AG9" t="n">
-        <v>221.7</v>
+        <v>429.33</v>
       </c>
       <c r="AH9" t="n">
-        <v>230.79</v>
+        <v>435.13</v>
       </c>
       <c r="AI9" t="n">
-        <v>239.89</v>
+        <v>440.94</v>
       </c>
       <c r="AJ9" t="n">
-        <v>248.99</v>
+        <v>446.74</v>
       </c>
     </row>
     <row r="10">
@@ -1730,88 +1730,88 @@
         <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>47.48</v>
+        <v>2549.23</v>
       </c>
       <c r="J10" t="n">
-        <v>47.48</v>
+        <v>2600.21</v>
       </c>
       <c r="K10" t="n">
-        <v>47.48</v>
+        <v>2651.2</v>
       </c>
       <c r="L10" t="n">
-        <v>54.22</v>
+        <v>2702.18</v>
       </c>
       <c r="M10" t="n">
-        <v>60.95</v>
+        <v>2753.17</v>
       </c>
       <c r="N10" t="n">
-        <v>67.69</v>
+        <v>2804.15</v>
       </c>
       <c r="O10" t="n">
-        <v>74.42</v>
+        <v>2855.14</v>
       </c>
       <c r="P10" t="n">
-        <v>81.15000000000001</v>
+        <v>2906.12</v>
       </c>
       <c r="Q10" t="n">
-        <v>88.8</v>
+        <v>2957.11</v>
       </c>
       <c r="R10" t="n">
-        <v>96.45999999999999</v>
+        <v>3008.09</v>
       </c>
       <c r="S10" t="n">
-        <v>104.11</v>
+        <v>3059.07</v>
       </c>
       <c r="T10" t="n">
-        <v>111.76</v>
+        <v>3110.06</v>
       </c>
       <c r="U10" t="n">
-        <v>119.41</v>
+        <v>3161.04</v>
       </c>
       <c r="V10" t="n">
-        <v>127.6</v>
+        <v>3212.03</v>
       </c>
       <c r="W10" t="n">
-        <v>135.78</v>
+        <v>3263.01</v>
       </c>
       <c r="X10" t="n">
-        <v>143.96</v>
+        <v>3314</v>
       </c>
       <c r="Y10" t="n">
-        <v>152.15</v>
+        <v>3364.98</v>
       </c>
       <c r="Z10" t="n">
-        <v>160.33</v>
+        <v>3415.97</v>
       </c>
       <c r="AA10" t="n">
-        <v>168.97</v>
+        <v>3466.95</v>
       </c>
       <c r="AB10" t="n">
-        <v>177.6</v>
+        <v>3517.94</v>
       </c>
       <c r="AC10" t="n">
-        <v>186.23</v>
+        <v>3568.92</v>
       </c>
       <c r="AD10" t="n">
-        <v>194.87</v>
+        <v>3619.91</v>
       </c>
       <c r="AE10" t="n">
-        <v>203.5</v>
+        <v>3670.89</v>
       </c>
       <c r="AF10" t="n">
-        <v>212.6</v>
+        <v>3721.87</v>
       </c>
       <c r="AG10" t="n">
-        <v>221.7</v>
+        <v>3772.86</v>
       </c>
       <c r="AH10" t="n">
-        <v>230.79</v>
+        <v>3823.84</v>
       </c>
       <c r="AI10" t="n">
-        <v>239.89</v>
+        <v>3874.83</v>
       </c>
       <c r="AJ10" t="n">
-        <v>248.99</v>
+        <v>3925.81</v>
       </c>
     </row>
     <row r="11">
@@ -1854,88 +1854,212 @@
         <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>18.94</v>
+        <v>302.39</v>
       </c>
       <c r="J11" t="n">
-        <v>18.94</v>
+        <v>308.44</v>
       </c>
       <c r="K11" t="n">
-        <v>18.94</v>
+        <v>314.49</v>
       </c>
       <c r="L11" t="n">
-        <v>18.94</v>
+        <v>320.54</v>
       </c>
       <c r="M11" t="n">
-        <v>18.94</v>
+        <v>326.58</v>
       </c>
       <c r="N11" t="n">
-        <v>18.94</v>
+        <v>332.63</v>
       </c>
       <c r="O11" t="n">
-        <v>18.94</v>
+        <v>338.68</v>
       </c>
       <c r="P11" t="n">
-        <v>18.94</v>
+        <v>344.73</v>
       </c>
       <c r="Q11" t="n">
-        <v>26.1</v>
+        <v>350.78</v>
       </c>
       <c r="R11" t="n">
-        <v>33.26</v>
+        <v>356.82</v>
       </c>
       <c r="S11" t="n">
-        <v>40.42</v>
+        <v>362.87</v>
       </c>
       <c r="T11" t="n">
-        <v>47.58</v>
+        <v>368.92</v>
       </c>
       <c r="U11" t="n">
-        <v>54.74</v>
+        <v>374.97</v>
       </c>
       <c r="V11" t="n">
-        <v>63.84</v>
+        <v>381.01</v>
       </c>
       <c r="W11" t="n">
-        <v>72.94</v>
+        <v>387.06</v>
       </c>
       <c r="X11" t="n">
-        <v>82.04000000000001</v>
+        <v>393.11</v>
       </c>
       <c r="Y11" t="n">
-        <v>91.14</v>
+        <v>399.16</v>
       </c>
       <c r="Z11" t="n">
-        <v>100.24</v>
+        <v>405.21</v>
       </c>
       <c r="AA11" t="n">
-        <v>110.25</v>
+        <v>411.25</v>
       </c>
       <c r="AB11" t="n">
-        <v>120.27</v>
+        <v>417.3</v>
       </c>
       <c r="AC11" t="n">
-        <v>130.28</v>
+        <v>423.35</v>
       </c>
       <c r="AD11" t="n">
-        <v>140.3</v>
+        <v>429.4</v>
       </c>
       <c r="AE11" t="n">
-        <v>150.31</v>
+        <v>435.45</v>
       </c>
       <c r="AF11" t="n">
-        <v>161.31</v>
+        <v>441.49</v>
       </c>
       <c r="AG11" t="n">
-        <v>172.3</v>
+        <v>447.54</v>
       </c>
       <c r="AH11" t="n">
-        <v>183.29</v>
+        <v>453.59</v>
       </c>
       <c r="AI11" t="n">
-        <v>194.29</v>
+        <v>459.64</v>
       </c>
       <c r="AJ11" t="n">
-        <v>205.28</v>
+        <v>465.68</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Demand</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ELCINDXX02</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Output demand of transmission lines in India</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>not needed</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>not needed</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>not needed</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>User defined</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" t="n">
+        <v>43.08</v>
+      </c>
+      <c r="J12" t="n">
+        <v>43.94</v>
+      </c>
+      <c r="K12" t="n">
+        <v>44.8</v>
+      </c>
+      <c r="L12" t="n">
+        <v>45.66</v>
+      </c>
+      <c r="M12" t="n">
+        <v>46.53</v>
+      </c>
+      <c r="N12" t="n">
+        <v>47.39</v>
+      </c>
+      <c r="O12" t="n">
+        <v>48.25</v>
+      </c>
+      <c r="P12" t="n">
+        <v>49.11</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>49.97</v>
+      </c>
+      <c r="R12" t="n">
+        <v>50.83</v>
+      </c>
+      <c r="S12" t="n">
+        <v>51.7</v>
+      </c>
+      <c r="T12" t="n">
+        <v>52.56</v>
+      </c>
+      <c r="U12" t="n">
+        <v>53.42</v>
+      </c>
+      <c r="V12" t="n">
+        <v>54.28</v>
+      </c>
+      <c r="W12" t="n">
+        <v>55.14</v>
+      </c>
+      <c r="X12" t="n">
+        <v>56</v>
+      </c>
+      <c r="Y12" t="n">
+        <v>56.87</v>
+      </c>
+      <c r="Z12" t="n">
+        <v>57.73</v>
+      </c>
+      <c r="AA12" t="n">
+        <v>58.59</v>
+      </c>
+      <c r="AB12" t="n">
+        <v>59.45</v>
+      </c>
+      <c r="AC12" t="n">
+        <v>60.31</v>
+      </c>
+      <c r="AD12" t="n">
+        <v>61.17</v>
+      </c>
+      <c r="AE12" t="n">
+        <v>62.03</v>
+      </c>
+      <c r="AF12" t="n">
+        <v>62.9</v>
+      </c>
+      <c r="AG12" t="n">
+        <v>63.76</v>
+      </c>
+      <c r="AH12" t="n">
+        <v>64.62</v>
+      </c>
+      <c r="AI12" t="n">
+        <v>65.48</v>
+      </c>
+      <c r="AJ12" t="n">
+        <v>66.34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>